<commit_message>
fix empty value assignment
</commit_message>
<xml_diff>
--- a/IfcManager.BL/Files/IfcManagerFiles/IFC parameters.xlsx
+++ b/IfcManager.BL/Files/IfcManagerFiles/IFC parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\supi\source\repos\IfcManager\IfcManager.BL\Files\IfcManagerFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19C27F49-7F58-49E4-A1D1-855DE69F1C76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B28E61C-C1D1-46E7-BCBB-62AACAB9941E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24105" yWindow="4080" windowWidth="30870" windowHeight="15345" tabRatio="745" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="38700" windowHeight="15345" tabRatio="745" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Properties" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7235" uniqueCount="4528">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7252" uniqueCount="4529">
   <si>
     <t>Data Type</t>
   </si>
@@ -13626,19 +13626,28 @@
   </si>
   <si>
     <t>RAMP-S</t>
+  </si>
+  <si>
+    <t>TUN.BAL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -13757,7 +13766,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -13852,70 +13861,88 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="7">
+  <cellStyleXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{FC528EF5-A6D0-4D13-9CE0-C50A2E61FD77}"/>
     <cellStyle name="Normal 3" xfId="2" xr:uid="{F3E263F6-78E8-4EA9-B859-F8D98F8BCA78}"/>
     <cellStyle name="Normal 3 2" xfId="5" xr:uid="{562A2998-00A4-431C-A5FE-06CC06040494}"/>
+    <cellStyle name="Normal 3 3" xfId="7" xr:uid="{94348558-55DC-4749-BCAB-781F42D46C86}"/>
     <cellStyle name="Normal 4" xfId="3" xr:uid="{4F4329F8-E4C2-4E19-BD86-CB810AFB9FBE}"/>
     <cellStyle name="Normal 4 2" xfId="6" xr:uid="{C1DA66DB-F815-47B4-BB2B-3901B21386C2}"/>
+    <cellStyle name="Normal 4 3" xfId="8" xr:uid="{647E405E-89F1-46B3-9D0F-7CADBB992D37}"/>
     <cellStyle name="Normal 5" xfId="4" xr:uid="{6DF54FAE-2483-4EEF-8D6C-A9E4680CE2F0}"/>
   </cellStyles>
   <dxfs count="9">
@@ -14116,8 +14143,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C8250F1A-5710-4EF4-AF6C-E853327E9515}" name="Table1" displayName="Table1" ref="A1:J166" totalsRowShown="0" headerRowDxfId="8">
-  <autoFilter ref="A1:J166" xr:uid="{C8250F1A-5710-4EF4-AF6C-E853327E9515}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C8250F1A-5710-4EF4-AF6C-E853327E9515}" name="Table1" displayName="Table1" ref="A1:J167" totalsRowShown="0" headerRowDxfId="8">
+  <autoFilter ref="A1:J167" xr:uid="{C8250F1A-5710-4EF4-AF6C-E853327E9515}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{7CD8FD0B-335F-4B2A-AB69-8C9EE375AC9F}" name="LocationRoot"/>
     <tableColumn id="2" xr3:uid="{E22D17F3-0FB5-4869-9840-DEB0FECC3DC6}" name="SubLocation"/>
@@ -14135,8 +14162,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{61158B8F-257E-4C05-AF7E-1081BDB1D7D4}" name="Table3" displayName="Table3" ref="A1:B56" totalsRowShown="0" tableBorderDxfId="7">
-  <autoFilter ref="A1:B56" xr:uid="{61158B8F-257E-4C05-AF7E-1081BDB1D7D4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{61158B8F-257E-4C05-AF7E-1081BDB1D7D4}" name="Table3" displayName="Table3" ref="A1:B63" totalsRowShown="0" tableBorderDxfId="7">
+  <autoFilter ref="A1:B63" xr:uid="{61158B8F-257E-4C05-AF7E-1081BDB1D7D4}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{4911EFDD-6DC1-4E8E-B65F-3B23EC4A6795}" name="LocationRoot" dataDxfId="6" dataCellStyle="Normal 2"/>
     <tableColumn id="2" xr3:uid="{4C9A0A65-1DCA-4EF9-BCD3-256BA43BE659}" name="SubLocation" dataDxfId="5" dataCellStyle="Normal 2"/>
@@ -14146,8 +14173,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{34C8FE38-B078-4F8C-9774-DDAA2832123B}" name="Table37" displayName="Table37" ref="A1:B165" totalsRowShown="0" tableBorderDxfId="4">
-  <autoFilter ref="A1:B165" xr:uid="{61158B8F-257E-4C05-AF7E-1081BDB1D7D4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{34C8FE38-B078-4F8C-9774-DDAA2832123B}" name="Table37" displayName="Table37" ref="A1:B166" totalsRowShown="0" tableBorderDxfId="4">
+  <autoFilter ref="A1:B166" xr:uid="{61158B8F-257E-4C05-AF7E-1081BDB1D7D4}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{A51CE557-8403-4E9D-AE1D-40B894898E7E}" name="TypeID" dataDxfId="3" dataCellStyle="Normal 2"/>
     <tableColumn id="2" xr3:uid="{798C78D9-BEA0-4284-A401-798B0EA1ECE7}" name="4DGroup" dataDxfId="2" dataCellStyle="Normal 2"/>
@@ -14671,7 +14698,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5E22C3A-731E-4720-A4F4-B02EE915C838}">
-  <dimension ref="A1:J166"/>
+  <dimension ref="A1:J167"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -16204,6 +16231,11 @@
     <row r="166" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D166" s="10" t="s">
         <v>4506</v>
+      </c>
+    </row>
+    <row r="167" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D167" s="10" t="s">
+        <v>4528</v>
       </c>
     </row>
   </sheetData>
@@ -39715,7 +39747,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6089D82B-CC96-4176-9A54-02325BF7F952}">
-  <dimension ref="A1:B56"/>
+  <dimension ref="A1:B63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -39788,10 +39820,10 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>140</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>152</v>
+        <v>126</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -39799,23 +39831,23 @@
         <v>140</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>150</v>
+        <v>140</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -39823,7 +39855,7 @@
         <v>127</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -39831,7 +39863,7 @@
         <v>127</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -39839,47 +39871,47 @@
         <v>127</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
-        <v>29</v>
+        <v>139</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>4463</v>
+        <v>152</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="10" t="s">
-        <v>29</v>
+        <v>139</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>4464</v>
+        <v>153</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="B20" s="10" t="s">
-        <v>4465</v>
+        <v>139</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -39887,7 +39919,7 @@
         <v>29</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>4466</v>
+        <v>4463</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -39895,7 +39927,7 @@
         <v>29</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>4467</v>
+        <v>4464</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -39903,7 +39935,7 @@
         <v>29</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>4468</v>
+        <v>4465</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -39911,39 +39943,39 @@
         <v>29</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>4469</v>
+        <v>4466</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
-        <v>115</v>
+        <v>29</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>4470</v>
+        <v>4467</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
-        <v>115</v>
+        <v>29</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>4471</v>
+        <v>4468</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
-        <v>115</v>
+        <v>29</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>4472</v>
+        <v>4469</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
-        <v>115</v>
-      </c>
-      <c r="B28" s="10" t="s">
-        <v>4473</v>
+        <v>29</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -39951,7 +39983,7 @@
         <v>115</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>4474</v>
+        <v>4470</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -39959,7 +39991,7 @@
         <v>115</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>4475</v>
+        <v>4471</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -39967,7 +39999,7 @@
         <v>115</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>4476</v>
+        <v>4472</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
@@ -39975,47 +40007,47 @@
         <v>115</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>4477</v>
+        <v>4473</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>4470</v>
+        <v>4474</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>4471</v>
+        <v>4475</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>4472</v>
+        <v>4476</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>4473</v>
+        <v>4477</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="B37" s="10" t="s">
-        <v>4474</v>
+        <v>115</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
@@ -40023,7 +40055,7 @@
         <v>116</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>4475</v>
+        <v>4470</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -40031,7 +40063,7 @@
         <v>116</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>4476</v>
+        <v>4471</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
@@ -40039,55 +40071,55 @@
         <v>116</v>
       </c>
       <c r="B40" s="10" t="s">
+        <v>4472</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="B41" s="10" t="s">
+        <v>4473</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="B42" s="10" t="s">
+        <v>4474</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="B43" s="10" t="s">
+        <v>4475</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="B44" s="10" t="s">
+        <v>4476</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="B45" s="10" t="s">
         <v>4477</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" s="24" t="s">
-        <v>4509</v>
-      </c>
-      <c r="B41" s="24" t="s">
-        <v>4512</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="24" t="s">
-        <v>4509</v>
-      </c>
-      <c r="B42" s="24" t="s">
-        <v>4513</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="24" t="s">
-        <v>4509</v>
-      </c>
-      <c r="B43" s="24" t="s">
-        <v>4514</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" s="24" t="s">
-        <v>4509</v>
-      </c>
-      <c r="B44" s="24" t="s">
-        <v>4515</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" s="24" t="s">
-        <v>4509</v>
-      </c>
-      <c r="B45" s="24" t="s">
-        <v>4516</v>
-      </c>
-    </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="24" t="s">
-        <v>4509</v>
-      </c>
-      <c r="B46" s="24" t="s">
-        <v>4517</v>
+      <c r="A46" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
@@ -40095,7 +40127,7 @@
         <v>4509</v>
       </c>
       <c r="B47" s="24" t="s">
-        <v>4518</v>
+        <v>4512</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
@@ -40103,7 +40135,7 @@
         <v>4509</v>
       </c>
       <c r="B48" s="24" t="s">
-        <v>4519</v>
+        <v>4513</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
@@ -40111,7 +40143,7 @@
         <v>4509</v>
       </c>
       <c r="B49" s="24" t="s">
-        <v>4520</v>
+        <v>4514</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
@@ -40119,7 +40151,7 @@
         <v>4509</v>
       </c>
       <c r="B50" s="24" t="s">
-        <v>4521</v>
+        <v>4515</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
@@ -40127,7 +40159,7 @@
         <v>4509</v>
       </c>
       <c r="B51" s="24" t="s">
-        <v>4522</v>
+        <v>4516</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
@@ -40135,7 +40167,7 @@
         <v>4509</v>
       </c>
       <c r="B52" s="24" t="s">
-        <v>4523</v>
+        <v>4517</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
@@ -40143,7 +40175,7 @@
         <v>4509</v>
       </c>
       <c r="B53" s="24" t="s">
-        <v>4524</v>
+        <v>4518</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
@@ -40151,7 +40183,7 @@
         <v>4509</v>
       </c>
       <c r="B54" s="24" t="s">
-        <v>4525</v>
+        <v>4519</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
@@ -40159,7 +40191,7 @@
         <v>4509</v>
       </c>
       <c r="B55" s="24" t="s">
-        <v>4526</v>
+        <v>4520</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
@@ -40167,7 +40199,63 @@
         <v>4509</v>
       </c>
       <c r="B56" s="24" t="s">
+        <v>4521</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" s="24" t="s">
+        <v>4509</v>
+      </c>
+      <c r="B57" s="24" t="s">
+        <v>4522</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" s="24" t="s">
+        <v>4509</v>
+      </c>
+      <c r="B58" s="24" t="s">
+        <v>4523</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" s="24" t="s">
+        <v>4509</v>
+      </c>
+      <c r="B59" s="24" t="s">
+        <v>4524</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" s="24" t="s">
+        <v>4509</v>
+      </c>
+      <c r="B60" s="24" t="s">
+        <v>4525</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" s="24" t="s">
+        <v>4509</v>
+      </c>
+      <c r="B61" s="24" t="s">
+        <v>4526</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" s="24" t="s">
+        <v>4509</v>
+      </c>
+      <c r="B62" s="24" t="s">
         <v>4527</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" s="22" t="s">
+        <v>4509</v>
+      </c>
+      <c r="B63" s="25" t="s">
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -40180,7 +40268,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{661F5D69-D337-4E34-A409-23B0595B8838}">
-  <dimension ref="A1:B165"/>
+  <dimension ref="A1:B166"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
@@ -40724,368 +40812,368 @@
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A68" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="B68" s="6" t="s">
-        <v>223</v>
+      <c r="A68" s="10" t="s">
+        <v>4528</v>
+      </c>
+      <c r="B68" s="10" t="s">
+        <v>4528</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B80" s="6" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B83" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B84" s="6" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B85" s="6" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B86" s="6" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B88" s="6" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B89" s="6" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B90" s="6" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B91" s="6" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B92" s="6" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B93" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B94" s="6" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B95" s="6" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B96" s="6" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B97" s="6" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B98" s="6" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B99" s="6" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B100" s="6" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B101" s="6" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B102" s="6" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B103" s="6" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B104" s="6" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B105" s="6" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B106" s="6" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B107" s="6" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B108" s="6" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B109" s="6" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B110" s="6" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B111" s="6" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="B112" s="6" t="s">
-        <v>4503</v>
+        <v>269</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B113" s="6" t="s">
         <v>4503</v>
@@ -41093,7 +41181,7 @@
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B114" s="6" t="s">
         <v>4503</v>
@@ -41101,7 +41189,7 @@
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B115" s="6" t="s">
         <v>4503</v>
@@ -41109,7 +41197,7 @@
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B116" s="6" t="s">
         <v>4503</v>
@@ -41117,7 +41205,7 @@
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B117" s="6" t="s">
         <v>4503</v>
@@ -41125,7 +41213,7 @@
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B118" s="6" t="s">
         <v>4503</v>
@@ -41133,7 +41221,7 @@
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B119" s="6" t="s">
         <v>4503</v>
@@ -41141,7 +41229,7 @@
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B120" s="6" t="s">
         <v>4503</v>
@@ -41149,7 +41237,7 @@
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B121" s="6" t="s">
         <v>4503</v>
@@ -41157,7 +41245,7 @@
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B122" s="6" t="s">
         <v>4503</v>
@@ -41165,7 +41253,7 @@
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B123" s="6" t="s">
         <v>4503</v>
@@ -41173,15 +41261,15 @@
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="B124" s="6" t="s">
-        <v>4504</v>
+        <v>4503</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B125" s="6" t="s">
         <v>4504</v>
@@ -41189,7 +41277,7 @@
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B126" s="6" t="s">
         <v>4504</v>
@@ -41197,7 +41285,7 @@
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B127" s="6" t="s">
         <v>4504</v>
@@ -41205,7 +41293,7 @@
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B128" s="6" t="s">
         <v>4504</v>
@@ -41213,7 +41301,7 @@
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B129" s="6" t="s">
         <v>4504</v>
@@ -41221,7 +41309,7 @@
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B130" s="6" t="s">
         <v>4504</v>
@@ -41229,7 +41317,7 @@
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B131" s="6" t="s">
         <v>4504</v>
@@ -41237,7 +41325,7 @@
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B132" s="6" t="s">
         <v>4504</v>
@@ -41245,7 +41333,7 @@
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B133" s="6" t="s">
         <v>4504</v>
@@ -41253,7 +41341,7 @@
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B134" s="6" t="s">
         <v>4504</v>
@@ -41261,7 +41349,7 @@
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B135" s="6" t="s">
         <v>4504</v>
@@ -41269,7 +41357,7 @@
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B136" s="6" t="s">
         <v>4504</v>
@@ -41277,7 +41365,7 @@
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B137" s="6" t="s">
         <v>4504</v>
@@ -41285,7 +41373,7 @@
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B138" s="6" t="s">
         <v>4504</v>
@@ -41293,7 +41381,7 @@
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B139" s="6" t="s">
         <v>4504</v>
@@ -41301,7 +41389,7 @@
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B140" s="6" t="s">
         <v>4504</v>
@@ -41309,7 +41397,7 @@
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B141" s="6" t="s">
         <v>4504</v>
@@ -41317,7 +41405,7 @@
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B142" s="6" t="s">
         <v>4504</v>
@@ -41325,7 +41413,7 @@
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B143" s="6" t="s">
         <v>4504</v>
@@ -41333,7 +41421,7 @@
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B144" s="6" t="s">
         <v>4504</v>
@@ -41341,7 +41429,7 @@
     </row>
     <row r="145" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B145" s="6" t="s">
         <v>4504</v>
@@ -41349,7 +41437,7 @@
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B146" s="6" t="s">
         <v>4504</v>
@@ -41357,153 +41445,161 @@
     </row>
     <row r="147" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B147" s="6" t="s">
-        <v>310</v>
+        <v>4504</v>
       </c>
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B148" s="6" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B149" s="6" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B150" s="6" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B151" s="6" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B152" s="6" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B153" s="6" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B154" s="6" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="155" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B155" s="6" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="156" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B156" s="6" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="157" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B157" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="158" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B158" s="6" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="159" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B159" s="6" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="160" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B160" s="6" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="161" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B161" s="6" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="162" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B162" s="6" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="163" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B163" s="6" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="164" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="B164" s="6" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A165" s="2" t="s">
         <v>327</v>
       </c>
-      <c r="B164" s="6" t="s">
+      <c r="B165" s="6" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A165" s="22" t="s">
+    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A166" s="22" t="s">
         <v>4506</v>
       </c>
-      <c r="B165" s="10" t="s">
+      <c r="B166" s="10" t="s">
         <v>4507</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update default excel settings
</commit_message>
<xml_diff>
--- a/IfcManager.BL/Files/IfcManagerFiles/IFC parameters.xlsx
+++ b/IfcManager.BL/Files/IfcManagerFiles/IFC parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\supi\source\repos\IfcManager\IfcManager.BL\Files\IfcManagerFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C51D1D39-F11D-47CB-ADBC-830A89270BA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{800E70F0-B0A2-455C-94B6-CFD62C3DC323}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30330" yWindow="1935" windowWidth="19455" windowHeight="15345" tabRatio="745" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="745" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Properties" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7252" uniqueCount="4529">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7466" uniqueCount="4735">
   <si>
     <t>Data Type</t>
   </si>
@@ -13629,6 +13629,624 @@
   </si>
   <si>
     <t>TUN.BAL</t>
+  </si>
+  <si>
+    <t>M&amp;E component ID</t>
+  </si>
+  <si>
+    <t>AB</t>
+  </si>
+  <si>
+    <t>AT</t>
+  </si>
+  <si>
+    <t>BC</t>
+  </si>
+  <si>
+    <t>BFD</t>
+  </si>
+  <si>
+    <t>BFI</t>
+  </si>
+  <si>
+    <t>BH</t>
+  </si>
+  <si>
+    <t>BM</t>
+  </si>
+  <si>
+    <t>BRO</t>
+  </si>
+  <si>
+    <t>BPB</t>
+  </si>
+  <si>
+    <t>BT</t>
+  </si>
+  <si>
+    <t>CSA</t>
+  </si>
+  <si>
+    <t>CSK</t>
+  </si>
+  <si>
+    <t>CSR</t>
+  </si>
+  <si>
+    <t>DA</t>
+  </si>
+  <si>
+    <t>DBK</t>
+  </si>
+  <si>
+    <t>DF</t>
+  </si>
+  <si>
+    <t>DKO</t>
+  </si>
+  <si>
+    <t>DS</t>
+  </si>
+  <si>
+    <t>DSW</t>
+  </si>
+  <si>
+    <t>DU</t>
+  </si>
+  <si>
+    <t>DYS</t>
+  </si>
+  <si>
+    <t>EBH</t>
+  </si>
+  <si>
+    <t>AFT</t>
+  </si>
+  <si>
+    <t>EEL</t>
+  </si>
+  <si>
+    <t>EFF</t>
+  </si>
+  <si>
+    <t>EGE</t>
+  </si>
+  <si>
+    <t>EIO</t>
+  </si>
+  <si>
+    <t>EKL</t>
+  </si>
+  <si>
+    <t>EKO</t>
+  </si>
+  <si>
+    <t>ELT</t>
+  </si>
+  <si>
+    <t>ENT</t>
+  </si>
+  <si>
+    <t>EVA</t>
+  </si>
+  <si>
+    <t>EVB</t>
+  </si>
+  <si>
+    <t>FKO</t>
+  </si>
+  <si>
+    <t>FLB</t>
+  </si>
+  <si>
+    <t>FLV</t>
+  </si>
+  <si>
+    <t>FLH</t>
+  </si>
+  <si>
+    <t>FLI</t>
+  </si>
+  <si>
+    <t>FLN</t>
+  </si>
+  <si>
+    <t>FLU</t>
+  </si>
+  <si>
+    <t>FO</t>
+  </si>
+  <si>
+    <t>FOB</t>
+  </si>
+  <si>
+    <t>FS</t>
+  </si>
+  <si>
+    <t>FIK</t>
+  </si>
+  <si>
+    <t>FTB</t>
+  </si>
+  <si>
+    <t>GAM</t>
+  </si>
+  <si>
+    <t>GB</t>
+  </si>
+  <si>
+    <t>HAI</t>
+  </si>
+  <si>
+    <t>HAS</t>
+  </si>
+  <si>
+    <t>HAU</t>
+  </si>
+  <si>
+    <t>HO</t>
+  </si>
+  <si>
+    <t>HPA</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>IDA</t>
+  </si>
+  <si>
+    <t>INC</t>
+  </si>
+  <si>
+    <t>IKF</t>
+  </si>
+  <si>
+    <t>IKV</t>
+  </si>
+  <si>
+    <t>IOM</t>
+  </si>
+  <si>
+    <t>KA</t>
+  </si>
+  <si>
+    <t>KFV</t>
+  </si>
+  <si>
+    <t>KG</t>
+  </si>
+  <si>
+    <t>KL</t>
+  </si>
+  <si>
+    <t>KFC</t>
+  </si>
+  <si>
+    <t>KNV</t>
+  </si>
+  <si>
+    <t>KOV</t>
+  </si>
+  <si>
+    <t>LSS</t>
+  </si>
+  <si>
+    <t>LEV</t>
+  </si>
+  <si>
+    <t>LIND</t>
+  </si>
+  <si>
+    <t>LGEN</t>
+  </si>
+  <si>
+    <t>LUD</t>
+  </si>
+  <si>
+    <t>LS</t>
+  </si>
+  <si>
+    <t>LSP</t>
+  </si>
+  <si>
+    <t>LUX</t>
+  </si>
+  <si>
+    <t>MAB</t>
+  </si>
+  <si>
+    <t>MAF</t>
+  </si>
+  <si>
+    <t>MAG</t>
+  </si>
+  <si>
+    <t>MAK</t>
+  </si>
+  <si>
+    <t>MAT</t>
+  </si>
+  <si>
+    <t>MAV</t>
+  </si>
+  <si>
+    <t>MBA</t>
+  </si>
+  <si>
+    <t>MEC</t>
+  </si>
+  <si>
+    <t>MIC</t>
+  </si>
+  <si>
+    <t>MST</t>
+  </si>
+  <si>
+    <t>MVB</t>
+  </si>
+  <si>
+    <t>MVK</t>
+  </si>
+  <si>
+    <t>MV</t>
+  </si>
+  <si>
+    <t>MVV</t>
+  </si>
+  <si>
+    <t>NC</t>
+  </si>
+  <si>
+    <t>NB</t>
+  </si>
+  <si>
+    <t>NEB</t>
+  </si>
+  <si>
+    <t>NEH</t>
+  </si>
+  <si>
+    <t>NEL</t>
+  </si>
+  <si>
+    <t>NH</t>
+  </si>
+  <si>
+    <t>NL</t>
+  </si>
+  <si>
+    <t>NOX</t>
+  </si>
+  <si>
+    <t>NVA</t>
+  </si>
+  <si>
+    <t>OKA</t>
+  </si>
+  <si>
+    <t>OPS</t>
+  </si>
+  <si>
+    <t>PBH</t>
+  </si>
+  <si>
+    <t>PD</t>
+  </si>
+  <si>
+    <t>PDV</t>
+  </si>
+  <si>
+    <t>PFI</t>
+  </si>
+  <si>
+    <t>PFU</t>
+  </si>
+  <si>
+    <t>PGE</t>
+  </si>
+  <si>
+    <t>PIR</t>
+  </si>
+  <si>
+    <t>PKB</t>
+  </si>
+  <si>
+    <t>PKL</t>
+  </si>
+  <si>
+    <t>PKO</t>
+  </si>
+  <si>
+    <t>POD</t>
+  </si>
+  <si>
+    <t>POV</t>
+  </si>
+  <si>
+    <t>POW</t>
+  </si>
+  <si>
+    <t>POA</t>
+  </si>
+  <si>
+    <t>PR</t>
+  </si>
+  <si>
+    <t>PRT</t>
+  </si>
+  <si>
+    <t>PSV</t>
+  </si>
+  <si>
+    <t>PI</t>
+  </si>
+  <si>
+    <t>PUA</t>
+  </si>
+  <si>
+    <t>RAA</t>
+  </si>
+  <si>
+    <t>PS</t>
+  </si>
+  <si>
+    <t>PT</t>
+  </si>
+  <si>
+    <t>PTI</t>
+  </si>
+  <si>
+    <t>PTU</t>
+  </si>
+  <si>
+    <t>PU</t>
+  </si>
+  <si>
+    <t>PVA</t>
+  </si>
+  <si>
+    <t>PVT</t>
+  </si>
+  <si>
+    <t>PVB</t>
+  </si>
+  <si>
+    <t>PVI</t>
+  </si>
+  <si>
+    <t>PVU</t>
+  </si>
+  <si>
+    <t>RAD</t>
+  </si>
+  <si>
+    <t>RED</t>
+  </si>
+  <si>
+    <t>REC</t>
+  </si>
+  <si>
+    <t>ROV</t>
+  </si>
+  <si>
+    <t>ROG</t>
+  </si>
+  <si>
+    <t>SC</t>
+  </si>
+  <si>
+    <t>SF</t>
+  </si>
+  <si>
+    <t>SIC</t>
+  </si>
+  <si>
+    <t>SIV</t>
+  </si>
+  <si>
+    <t>SG</t>
+  </si>
+  <si>
+    <t>SKO</t>
+  </si>
+  <si>
+    <t>SNS</t>
+  </si>
+  <si>
+    <t>SMB</t>
+  </si>
+  <si>
+    <t>SMG</t>
+  </si>
+  <si>
+    <t>SMI</t>
+  </si>
+  <si>
+    <t>SMP</t>
+  </si>
+  <si>
+    <t>SMR</t>
+  </si>
+  <si>
+    <t>SMU</t>
+  </si>
+  <si>
+    <t>SOS</t>
+  </si>
+  <si>
+    <t>SPB</t>
+  </si>
+  <si>
+    <t>SR</t>
+  </si>
+  <si>
+    <t>STA</t>
+  </si>
+  <si>
+    <t>STO</t>
+  </si>
+  <si>
+    <t>SVR</t>
+  </si>
+  <si>
+    <t>TBE</t>
+  </si>
+  <si>
+    <t>TBI</t>
+  </si>
+  <si>
+    <t>TBU</t>
+  </si>
+  <si>
+    <t>TD</t>
+  </si>
+  <si>
+    <t>TDP</t>
+  </si>
+  <si>
+    <t>TDF</t>
+  </si>
+  <si>
+    <t>TEG</t>
+  </si>
+  <si>
+    <t>TF</t>
+  </si>
+  <si>
+    <t>TFG</t>
+  </si>
+  <si>
+    <t>TFI</t>
+  </si>
+  <si>
+    <t>TI</t>
+  </si>
+  <si>
+    <t>TKA</t>
+  </si>
+  <si>
+    <t>TR</t>
+  </si>
+  <si>
+    <t>TND</t>
+  </si>
+  <si>
+    <t>TRU</t>
+  </si>
+  <si>
+    <t>TRD</t>
+  </si>
+  <si>
+    <t>TT</t>
+  </si>
+  <si>
+    <t>TU</t>
+  </si>
+  <si>
+    <t>TUD</t>
+  </si>
+  <si>
+    <t>UPS</t>
+  </si>
+  <si>
+    <t>UT</t>
+  </si>
+  <si>
+    <t>VAC</t>
+  </si>
+  <si>
+    <t>VAE</t>
+  </si>
+  <si>
+    <t>VAR</t>
+  </si>
+  <si>
+    <t>VAV</t>
+  </si>
+  <si>
+    <t>VAT</t>
+  </si>
+  <si>
+    <t>VBX</t>
+  </si>
+  <si>
+    <t>VD</t>
+  </si>
+  <si>
+    <t>VE</t>
+  </si>
+  <si>
+    <t>VEI</t>
+  </si>
+  <si>
+    <t>VER</t>
+  </si>
+  <si>
+    <t>VEU</t>
+  </si>
+  <si>
+    <t>VFI</t>
+  </si>
+  <si>
+    <t>VIK</t>
+  </si>
+  <si>
+    <t>VIP</t>
+  </si>
+  <si>
+    <t>VIM</t>
+  </si>
+  <si>
+    <t>VK</t>
+  </si>
+  <si>
+    <t>VM</t>
+  </si>
+  <si>
+    <t>VMO</t>
+  </si>
+  <si>
+    <t>VS</t>
+  </si>
+  <si>
+    <t>VT</t>
+  </si>
+  <si>
+    <t>VT1</t>
+  </si>
+  <si>
+    <t>VT2</t>
+  </si>
+  <si>
+    <t>VIH</t>
+  </si>
+  <si>
+    <t>VIR</t>
+  </si>
+  <si>
+    <t>VMS</t>
+  </si>
+  <si>
+    <t>VOT</t>
+  </si>
+  <si>
+    <t>VSLS</t>
+  </si>
+  <si>
+    <t>VUR</t>
+  </si>
+  <si>
+    <t>VVF</t>
+  </si>
+  <si>
+    <t>VVX</t>
+  </si>
+  <si>
+    <t>VZ</t>
+  </si>
+  <si>
+    <t>AA</t>
   </si>
 </sst>
 </file>
@@ -13886,7 +14504,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFill="1" applyBorder="1"/>
@@ -13933,6 +14551,7 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13946,6 +14565,23 @@
     <cellStyle name="Normal 5" xfId="4" xr:uid="{6DF54FAE-2483-4EEF-8D6C-A9E4680CE2F0}"/>
   </cellStyles>
   <dxfs count="9">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -14100,23 +14736,6 @@
         </bottom>
       </border>
     </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -14131,8 +14750,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E01B3177-0B4D-4D90-AD21-322A353B9D10}" name="Table2" displayName="Table2" ref="A1:C19" totalsRowShown="0">
-  <autoFilter ref="A1:C19" xr:uid="{E01B3177-0B4D-4D90-AD21-322A353B9D10}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E01B3177-0B4D-4D90-AD21-322A353B9D10}" name="Table2" displayName="Table2" ref="A1:C20" totalsRowShown="0">
+  <autoFilter ref="A1:C20" xr:uid="{E01B3177-0B4D-4D90-AD21-322A353B9D10}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{3761E3A8-6DA3-4AC8-9E60-9889E5200835}" name="Property Set Name"/>
     <tableColumn id="2" xr3:uid="{33F19375-2CEB-4E6B-994E-E4F9F9266E3A}" name="Property Name"/>
@@ -14143,9 +14762,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C8250F1A-5710-4EF4-AF6C-E853327E9515}" name="Table1" displayName="Table1" ref="A1:J167" totalsRowShown="0" headerRowDxfId="8">
-  <autoFilter ref="A1:J167" xr:uid="{C8250F1A-5710-4EF4-AF6C-E853327E9515}"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C8250F1A-5710-4EF4-AF6C-E853327E9515}" name="Table1" displayName="Table1" ref="A1:K211" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:K211" xr:uid="{C8250F1A-5710-4EF4-AF6C-E853327E9515}"/>
+  <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{7CD8FD0B-335F-4B2A-AB69-8C9EE375AC9F}" name="LocationRoot"/>
     <tableColumn id="2" xr3:uid="{E22D17F3-0FB5-4869-9840-DEB0FECC3DC6}" name="SubLocation"/>
     <tableColumn id="3" xr3:uid="{A82C31E6-FA85-4B9B-BA5F-B0D187D6F06D}" name="OrientationID"/>
@@ -14156,28 +14775,29 @@
     <tableColumn id="8" xr3:uid="{3CEB9467-2E3D-4F1E-A4A4-9C65476A8AE5}" name="WorkStep"/>
     <tableColumn id="9" xr3:uid="{B8A60227-91EF-4766-98CB-A9DA957FC5D0}" name="ConstructionPhase"/>
     <tableColumn id="10" xr3:uid="{C2227E0B-2BFC-41C1-97BD-D33A930BE581}" name="AccessConstraint"/>
+    <tableColumn id="11" xr3:uid="{023A7533-A195-4DCA-AC34-BD6926A74239}" name="M&amp;E component ID" dataCellStyle="Normal 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{61158B8F-257E-4C05-AF7E-1081BDB1D7D4}" name="Table3" displayName="Table3" ref="A1:B63" totalsRowShown="0" tableBorderDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{61158B8F-257E-4C05-AF7E-1081BDB1D7D4}" name="Table3" displayName="Table3" ref="A1:B63" totalsRowShown="0" tableBorderDxfId="8">
   <autoFilter ref="A1:B63" xr:uid="{61158B8F-257E-4C05-AF7E-1081BDB1D7D4}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{4911EFDD-6DC1-4E8E-B65F-3B23EC4A6795}" name="LocationRoot" dataDxfId="6" dataCellStyle="Normal 2"/>
-    <tableColumn id="2" xr3:uid="{4C9A0A65-1DCA-4EF9-BCD3-256BA43BE659}" name="SubLocation" dataDxfId="5" dataCellStyle="Normal 2"/>
+    <tableColumn id="1" xr3:uid="{4911EFDD-6DC1-4E8E-B65F-3B23EC4A6795}" name="LocationRoot" dataDxfId="7" dataCellStyle="Normal 2"/>
+    <tableColumn id="2" xr3:uid="{4C9A0A65-1DCA-4EF9-BCD3-256BA43BE659}" name="SubLocation" dataDxfId="6" dataCellStyle="Normal 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{34C8FE38-B078-4F8C-9774-DDAA2832123B}" name="Table37" displayName="Table37" ref="A1:B166" totalsRowShown="0" tableBorderDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{34C8FE38-B078-4F8C-9774-DDAA2832123B}" name="Table37" displayName="Table37" ref="A1:B166" totalsRowShown="0" tableBorderDxfId="5">
   <autoFilter ref="A1:B166" xr:uid="{61158B8F-257E-4C05-AF7E-1081BDB1D7D4}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{A51CE557-8403-4E9D-AE1D-40B894898E7E}" name="TypeID" dataDxfId="3" dataCellStyle="Normal 2"/>
-    <tableColumn id="2" xr3:uid="{798C78D9-BEA0-4284-A401-798B0EA1ECE7}" name="4DGroup" dataDxfId="2" dataCellStyle="Normal 2"/>
+    <tableColumn id="1" xr3:uid="{A51CE557-8403-4E9D-AE1D-40B894898E7E}" name="TypeID" dataDxfId="4" dataCellStyle="Normal 2"/>
+    <tableColumn id="2" xr3:uid="{798C78D9-BEA0-4284-A401-798B0EA1ECE7}" name="4DGroup" dataDxfId="3" dataCellStyle="Normal 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -14187,8 +14807,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{B0F2E238-E1C5-400D-B944-80181B90F609}" name="Table4" displayName="Table4" ref="A1:D3" totalsRowShown="0">
   <autoFilter ref="A1:D3" xr:uid="{B0F2E238-E1C5-400D-B944-80181B90F609}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{A0CDC16A-3706-47C9-9E77-C6678E0326C3}" name="Source Property Name" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{4BC30CBE-C5F5-4A85-8E76-B531F3265739}" name="Target Property Name" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{A0CDC16A-3706-47C9-9E77-C6678E0326C3}" name="Source Property Name" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{4BC30CBE-C5F5-4A85-8E76-B531F3265739}" name="Target Property Name" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{DF1EFB03-B9BD-43A3-A819-4FC3E2BCCDD0}" name="Function"/>
     <tableColumn id="4" xr3:uid="{F590C646-6614-44AA-8C48-74C4100AC227}" name="Value"/>
   </tableColumns>
@@ -14470,7 +15090,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.85546875" bestFit="1" customWidth="1"/>
@@ -14591,10 +15211,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>4483</v>
+        <v>4482</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
+        <v>4529</v>
       </c>
       <c r="C11" t="s">
         <v>6</v>
@@ -14605,7 +15225,7 @@
         <v>4483</v>
       </c>
       <c r="B12" t="s">
-        <v>4484</v>
+        <v>15</v>
       </c>
       <c r="C12" t="s">
         <v>6</v>
@@ -14616,7 +15236,7 @@
         <v>4483</v>
       </c>
       <c r="B13" t="s">
-        <v>17</v>
+        <v>4484</v>
       </c>
       <c r="C13" t="s">
         <v>6</v>
@@ -14627,7 +15247,7 @@
         <v>4483</v>
       </c>
       <c r="B14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C14" t="s">
         <v>6</v>
@@ -14638,7 +15258,7 @@
         <v>4483</v>
       </c>
       <c r="B15" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C15" t="s">
         <v>6</v>
@@ -14649,10 +15269,10 @@
         <v>4483</v>
       </c>
       <c r="B16" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C16" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -14660,10 +15280,10 @@
         <v>4483</v>
       </c>
       <c r="B17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C17" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -14671,10 +15291,10 @@
         <v>4483</v>
       </c>
       <c r="B18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C18" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -14682,9 +15302,20 @@
         <v>4483</v>
       </c>
       <c r="B19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>4483</v>
+      </c>
+      <c r="B20" t="s">
         <v>22</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -14698,7 +15329,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5E22C3A-731E-4720-A4F4-B02EE915C838}">
-  <dimension ref="A1:J167"/>
+  <dimension ref="A1:K211"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -14711,9 +15342,10 @@
     <col min="8" max="8" width="15.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="20.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17.5703125" customWidth="1"/>
+    <col min="11" max="11" width="22.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
         <v>9</v>
       </c>
@@ -14744,8 +15376,11 @@
       <c r="J1" s="17" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K1" s="18" t="s">
+        <v>4529</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4505</v>
       </c>
@@ -14776,8 +15411,11 @@
       <c r="J2" t="s">
         <v>4488</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K2" s="10" t="s">
+        <v>4530</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>23</v>
       </c>
@@ -14805,8 +15443,11 @@
       <c r="J3" t="s">
         <v>4490</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K3" s="10" t="s">
+        <v>4531</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>24</v>
       </c>
@@ -14834,8 +15475,11 @@
       <c r="J4" t="s">
         <v>4489</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K4" s="10" t="s">
+        <v>4532</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>25</v>
       </c>
@@ -14860,8 +15504,11 @@
       <c r="H5" t="s">
         <v>361</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K5" s="10" t="s">
+        <v>4533</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>26</v>
       </c>
@@ -14883,8 +15530,11 @@
       <c r="H6" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K6" s="10" t="s">
+        <v>4534</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>27</v>
       </c>
@@ -14906,8 +15556,11 @@
       <c r="H7" t="s">
         <v>363</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K7" s="10" t="s">
+        <v>4535</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>28</v>
       </c>
@@ -14923,8 +15576,11 @@
       <c r="F8" s="10" t="s">
         <v>356</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K8" s="10" t="s">
+        <v>4536</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>29</v>
       </c>
@@ -14940,8 +15596,11 @@
       <c r="F9" s="10" t="s">
         <v>357</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K9" s="10" t="s">
+        <v>4537</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>30</v>
       </c>
@@ -14957,8 +15616,11 @@
       <c r="F10" s="10" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K10" s="10" t="s">
+        <v>4538</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>31</v>
       </c>
@@ -14974,8 +15636,11 @@
       <c r="F11" s="10" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K11" s="10" t="s">
+        <v>4539</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>32</v>
       </c>
@@ -14991,8 +15656,11 @@
       <c r="F12" s="10" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K12" s="10" t="s">
+        <v>4540</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>33</v>
       </c>
@@ -15008,8 +15676,11 @@
       <c r="F13" s="10" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K13" s="10" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>34</v>
       </c>
@@ -15025,8 +15696,11 @@
       <c r="F14" s="10" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K14" s="10" t="s">
+        <v>4541</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>35</v>
       </c>
@@ -15042,8 +15716,11 @@
       <c r="F15" s="10" t="s">
         <v>284</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K15" s="10" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>36</v>
       </c>
@@ -15059,8 +15736,11 @@
       <c r="F16" s="10" t="s">
         <v>309</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="K16" s="10" t="s">
+        <v>4542</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>37</v>
       </c>
@@ -15073,8 +15753,11 @@
       <c r="E17" s="10" t="s">
         <v>343</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="K17" s="10" t="s">
+        <v>4543</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>38</v>
       </c>
@@ -15087,8 +15770,11 @@
       <c r="E18" s="10" t="s">
         <v>344</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="K18" s="10" t="s">
+        <v>4544</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>39</v>
       </c>
@@ -15101,8 +15787,11 @@
       <c r="E19" s="10" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="K19" s="10" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>40</v>
       </c>
@@ -15115,8 +15804,11 @@
       <c r="E20" s="10" t="s">
         <v>346</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="K20" s="10" t="s">
+        <v>4545</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>41</v>
       </c>
@@ -15126,8 +15818,11 @@
       <c r="D21" s="10" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="K21" s="10" t="s">
+        <v>4546</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>42</v>
       </c>
@@ -15137,8 +15832,11 @@
       <c r="D22" s="10" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="K22" s="10" t="s">
+        <v>4547</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>43</v>
       </c>
@@ -15148,8 +15846,11 @@
       <c r="D23" s="10" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="K23" s="10" t="s">
+        <v>4548</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>44</v>
       </c>
@@ -15159,8 +15860,11 @@
       <c r="D24" s="10" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="K24" s="10" t="s">
+        <v>4549</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>45</v>
       </c>
@@ -15170,8 +15874,11 @@
       <c r="D25" s="10" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="K25" s="10" t="s">
+        <v>4550</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>46</v>
       </c>
@@ -15181,8 +15888,11 @@
       <c r="D26" s="10" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="K26" s="10" t="s">
+        <v>4551</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>47</v>
       </c>
@@ -15192,8 +15902,11 @@
       <c r="D27" s="10" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="K27" s="10" t="s">
+        <v>4552</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>48</v>
       </c>
@@ -15203,8 +15916,11 @@
       <c r="D28" s="10" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="K28" s="10" t="s">
+        <v>4553</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>49</v>
       </c>
@@ -15214,8 +15930,11 @@
       <c r="D29" s="10" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="K29" s="10" t="s">
+        <v>4554</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>50</v>
       </c>
@@ -15225,8 +15944,11 @@
       <c r="D30" s="10" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="K30" s="10" t="s">
+        <v>4555</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>51</v>
       </c>
@@ -15236,8 +15958,11 @@
       <c r="D31" s="10" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="K31" s="10" t="s">
+        <v>4556</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>52</v>
       </c>
@@ -15247,8 +15972,11 @@
       <c r="D32" s="10" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K32" s="10" t="s">
+        <v>4557</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>53</v>
       </c>
@@ -15258,8 +15986,11 @@
       <c r="D33" s="10" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K33" s="10" t="s">
+        <v>4558</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>54</v>
       </c>
@@ -15269,8 +16000,11 @@
       <c r="D34" s="10" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K34" s="10" t="s">
+        <v>4559</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>55</v>
       </c>
@@ -15280,8 +16014,11 @@
       <c r="D35" s="10" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K35" s="10" t="s">
+        <v>4560</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>56</v>
       </c>
@@ -15291,8 +16028,11 @@
       <c r="D36" s="10" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K36" s="10" t="s">
+        <v>4561</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>57</v>
       </c>
@@ -15302,8 +16042,11 @@
       <c r="D37" s="10" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K37" s="10" t="s">
+        <v>4562</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>58</v>
       </c>
@@ -15313,8 +16056,11 @@
       <c r="D38" s="10" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K38" s="10" t="s">
+        <v>4563</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>59</v>
       </c>
@@ -15324,8 +16070,11 @@
       <c r="D39" s="10" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K39" s="10" t="s">
+        <v>4564</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>60</v>
       </c>
@@ -15335,8 +16084,11 @@
       <c r="D40" s="10" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K40" s="10" t="s">
+        <v>4565</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>61</v>
       </c>
@@ -15346,896 +16098,1541 @@
       <c r="D41" s="10" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K41" s="10" t="s">
+        <v>4566</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>62</v>
       </c>
       <c r="D42" s="10" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K42" s="10" t="s">
+        <v>4567</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>63</v>
       </c>
       <c r="D43" s="10" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K43" s="10" t="s">
+        <v>4568</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>64</v>
       </c>
       <c r="D44" s="10" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K44" s="10" t="s">
+        <v>4569</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>65</v>
       </c>
       <c r="D45" s="10" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K45" s="10" t="s">
+        <v>4570</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>66</v>
       </c>
       <c r="D46" s="10" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K46" s="10" t="s">
+        <v>4571</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>67</v>
       </c>
       <c r="D47" s="10" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K47" s="10" t="s">
+        <v>4572</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>68</v>
       </c>
       <c r="D48" s="10" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K48" s="10" t="s">
+        <v>4573</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>69</v>
       </c>
       <c r="D49" s="10" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K49" s="10" t="s">
+        <v>4574</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D50" s="10" t="s">
         <v>208</v>
       </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K50" s="10" t="s">
+        <v>4575</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>71</v>
       </c>
       <c r="D51" s="10" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K51" s="10" t="s">
+        <v>4576</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>72</v>
       </c>
       <c r="D52" s="10" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K52" s="10" t="s">
+        <v>4577</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>73</v>
       </c>
       <c r="D53" s="10" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K53" s="10" t="s">
+        <v>4578</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>74</v>
       </c>
       <c r="D54" s="10" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K54" s="10" t="s">
+        <v>4579</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>75</v>
       </c>
       <c r="D55" s="10" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K55" s="10" t="s">
+        <v>4580</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>76</v>
       </c>
       <c r="D56" s="10" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K56" s="10" t="s">
+        <v>4581</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>77</v>
       </c>
       <c r="D57" s="10" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K57" s="10" t="s">
+        <v>4582</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>78</v>
       </c>
       <c r="D58" s="10" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K58" s="10" t="s">
+        <v>4583</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>79</v>
       </c>
       <c r="D59" s="10" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K59" s="10" t="s">
+        <v>4584</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D60" s="10" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K60" s="10" t="s">
+        <v>4585</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>81</v>
       </c>
       <c r="D61" s="10" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K61" s="10" t="s">
+        <v>4586</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>82</v>
       </c>
       <c r="D62" s="10" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K62" s="10" t="s">
+        <v>4587</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>83</v>
       </c>
       <c r="D63" s="10" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K63" s="10" t="s">
+        <v>4588</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>84</v>
       </c>
       <c r="D64" s="10" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K64" s="10" t="s">
+        <v>4589</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>85</v>
       </c>
       <c r="D65" s="10" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K65" s="10" t="s">
+        <v>4590</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>86</v>
       </c>
       <c r="D66" s="10" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K66" s="10" t="s">
+        <v>4591</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>87</v>
       </c>
       <c r="D67" s="10" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K67" s="10" t="s">
+        <v>4592</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>88</v>
       </c>
       <c r="D68" s="10" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K68" s="10" t="s">
+        <v>4593</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>89</v>
       </c>
       <c r="D69" s="10" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K69" s="10" t="s">
+        <v>4594</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>90</v>
       </c>
       <c r="D70" s="10" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K70" s="10" t="s">
+        <v>4595</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>91</v>
       </c>
       <c r="D71" s="10" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K71" s="10" t="s">
+        <v>4596</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>92</v>
       </c>
       <c r="D72" s="10" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K72" s="10" t="s">
+        <v>4597</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>93</v>
       </c>
       <c r="D73" s="10" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K73" s="10" t="s">
+        <v>4598</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>94</v>
       </c>
       <c r="D74" s="10" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K74" s="10" t="s">
+        <v>4599</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>95</v>
       </c>
       <c r="D75" s="10" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K75" s="10" t="s">
+        <v>4600</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>96</v>
       </c>
       <c r="D76" s="10" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K76" s="10" t="s">
+        <v>4601</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>97</v>
       </c>
       <c r="D77" s="10" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K77" s="10" t="s">
+        <v>4602</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>98</v>
       </c>
       <c r="D78" s="10" t="s">
         <v>233</v>
       </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K78" s="10" t="s">
+        <v>4603</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>99</v>
       </c>
       <c r="D79" s="10" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K79" s="10" t="s">
+        <v>4604</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>100</v>
       </c>
       <c r="D80" s="10" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K80" s="10" t="s">
+        <v>4605</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>101</v>
       </c>
       <c r="D81" s="10" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K81" s="10" t="s">
+        <v>4606</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>102</v>
       </c>
       <c r="D82" s="10" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K82" s="10" t="s">
+        <v>4607</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>103</v>
       </c>
       <c r="D83" s="10" t="s">
         <v>238</v>
       </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K83" s="10" t="s">
+        <v>4608</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>104</v>
       </c>
       <c r="D84" s="10" t="s">
         <v>239</v>
       </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K84" s="10" t="s">
+        <v>4609</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>105</v>
       </c>
       <c r="D85" s="10" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K85" s="10" t="s">
+        <v>4610</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>106</v>
       </c>
       <c r="D86" s="10" t="s">
         <v>241</v>
       </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K86" s="10" t="s">
+        <v>4611</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>107</v>
       </c>
       <c r="D87" s="10" t="s">
         <v>242</v>
       </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K87" s="10" t="s">
+        <v>4612</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>108</v>
       </c>
       <c r="D88" s="10" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K88" s="10" t="s">
+        <v>4613</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>109</v>
       </c>
       <c r="D89" s="10" t="s">
         <v>245</v>
       </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K89" s="10" t="s">
+        <v>4614</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>110</v>
       </c>
       <c r="D90" s="10" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K90" s="10" t="s">
+        <v>4615</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>111</v>
       </c>
       <c r="D91" s="10" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K91" s="10" t="s">
+        <v>4616</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
         <v>112</v>
       </c>
       <c r="D92" s="10" t="s">
         <v>248</v>
       </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K92" s="10" t="s">
+        <v>4617</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>113</v>
       </c>
       <c r="D93" s="10" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K93" s="10" t="s">
+        <v>4618</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
         <v>114</v>
       </c>
       <c r="D94" s="10" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K94" s="10" t="s">
+        <v>4619</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>115</v>
       </c>
       <c r="D95" s="10" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K95" s="10" t="s">
+        <v>4620</v>
+      </c>
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>116</v>
       </c>
       <c r="D96" s="10" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K96" s="10" t="s">
+        <v>4621</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
         <v>117</v>
       </c>
       <c r="D97" s="10" t="s">
         <v>254</v>
       </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K97" s="10" t="s">
+        <v>4622</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
         <v>118</v>
       </c>
       <c r="D98" s="10" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K98" s="10" t="s">
+        <v>4623</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>119</v>
       </c>
       <c r="D99" s="10" t="s">
         <v>256</v>
       </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K99" s="10" t="s">
+        <v>4624</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
         <v>120</v>
       </c>
       <c r="D100" s="10" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K100" s="10" t="s">
+        <v>4625</v>
+      </c>
+    </row>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>121</v>
       </c>
       <c r="D101" s="10" t="s">
         <v>258</v>
       </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K101" s="10" t="s">
+        <v>4626</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
         <v>122</v>
       </c>
       <c r="D102" s="10" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K102" s="10" t="s">
+        <v>4627</v>
+      </c>
+    </row>
+    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>123</v>
       </c>
       <c r="D103" s="10" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K103" s="10" t="s">
+        <v>4628</v>
+      </c>
+    </row>
+    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>124</v>
       </c>
       <c r="D104" s="10" t="s">
         <v>261</v>
       </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K104" s="10" t="s">
+        <v>4629</v>
+      </c>
+    </row>
+    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>125</v>
       </c>
       <c r="D105" s="10" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K105" s="10" t="s">
+        <v>4630</v>
+      </c>
+    </row>
+    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
         <v>4509</v>
       </c>
       <c r="D106" s="10" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K106" s="10" t="s">
+        <v>4631</v>
+      </c>
+    </row>
+    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>127</v>
       </c>
       <c r="D107" s="10" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K107" s="10" t="s">
+        <v>4632</v>
+      </c>
+    </row>
+    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
         <v>126</v>
       </c>
       <c r="D108" s="10" t="s">
         <v>266</v>
       </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K108" s="10" t="s">
+        <v>4633</v>
+      </c>
+    </row>
+    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
         <v>128</v>
       </c>
       <c r="D109" s="10" t="s">
         <v>267</v>
       </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K109" s="10" t="s">
+        <v>4634</v>
+      </c>
+    </row>
+    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>4510</v>
       </c>
       <c r="D110" s="10" t="s">
         <v>268</v>
       </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K110" s="10" t="s">
+        <v>4635</v>
+      </c>
+    </row>
+    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>4511</v>
       </c>
       <c r="D111" s="10" t="s">
         <v>269</v>
       </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K111" s="10" t="s">
+        <v>4636</v>
+      </c>
+    </row>
+    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
         <v>129</v>
       </c>
       <c r="D112" s="10" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K112" s="10" t="s">
+        <v>4637</v>
+      </c>
+    </row>
+    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
         <v>130</v>
       </c>
       <c r="D113" s="10" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K113" s="10" t="s">
+        <v>4638</v>
+      </c>
+    </row>
+    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
         <v>131</v>
       </c>
       <c r="D114" s="10" t="s">
         <v>273</v>
       </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K114" s="10" t="s">
+        <v>4639</v>
+      </c>
+    </row>
+    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
         <v>132</v>
       </c>
       <c r="D115" s="10" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K115" s="10" t="s">
+        <v>4640</v>
+      </c>
+    </row>
+    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
         <v>133</v>
       </c>
       <c r="D116" s="10" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K116" s="10" t="s">
+        <v>4641</v>
+      </c>
+    </row>
+    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
         <v>134</v>
       </c>
       <c r="D117" s="10" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K117" s="10" t="s">
+        <v>4642</v>
+      </c>
+    </row>
+    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>135</v>
       </c>
       <c r="D118" s="10" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K118" s="10" t="s">
+        <v>4643</v>
+      </c>
+    </row>
+    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
         <v>136</v>
       </c>
       <c r="D119" s="10" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K119" s="10" t="s">
+        <v>4644</v>
+      </c>
+    </row>
+    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
         <v>137</v>
       </c>
       <c r="D120" s="10" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K120" s="10" t="s">
+        <v>4645</v>
+      </c>
+    </row>
+    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
         <v>138</v>
       </c>
       <c r="D121" s="10" t="s">
         <v>281</v>
       </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K121" s="10" t="s">
+        <v>4646</v>
+      </c>
+    </row>
+    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
         <v>139</v>
       </c>
       <c r="D122" s="10" t="s">
         <v>282</v>
       </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K122" s="10" t="s">
+        <v>4647</v>
+      </c>
+    </row>
+    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
         <v>140</v>
       </c>
       <c r="D123" s="10" t="s">
         <v>283</v>
       </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K123" s="10" t="s">
+        <v>4648</v>
+      </c>
+    </row>
+    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
         <v>141</v>
       </c>
       <c r="D124" s="10" t="s">
         <v>285</v>
       </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K124" s="10" t="s">
+        <v>4649</v>
+      </c>
+    </row>
+    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
         <v>142</v>
       </c>
       <c r="D125" s="10" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K125" s="10" t="s">
+        <v>4650</v>
+      </c>
+    </row>
+    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
         <v>143</v>
       </c>
       <c r="D126" s="10" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K126" s="10" t="s">
+        <v>4651</v>
+      </c>
+    </row>
+    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A127" s="4" t="s">
         <v>144</v>
       </c>
       <c r="D127" s="10" t="s">
         <v>288</v>
       </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="K127" s="10" t="s">
+        <v>4652</v>
+      </c>
+    </row>
+    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>145</v>
       </c>
       <c r="D128" s="10" t="s">
         <v>289</v>
       </c>
-    </row>
-    <row r="129" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K128" s="10" t="s">
+        <v>4653</v>
+      </c>
+    </row>
+    <row r="129" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D129" s="10" t="s">
         <v>290</v>
       </c>
-    </row>
-    <row r="130" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K129" s="10" t="s">
+        <v>4637</v>
+      </c>
+    </row>
+    <row r="130" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D130" s="10" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="131" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K130" s="10" t="s">
+        <v>4654</v>
+      </c>
+    </row>
+    <row r="131" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D131" s="10" t="s">
         <v>292</v>
       </c>
-    </row>
-    <row r="132" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K131" s="10" t="s">
+        <v>4655</v>
+      </c>
+    </row>
+    <row r="132" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D132" s="10" t="s">
         <v>293</v>
       </c>
-    </row>
-    <row r="133" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K132" s="10" t="s">
+        <v>4656</v>
+      </c>
+    </row>
+    <row r="133" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D133" s="10" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="134" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K133" s="10" t="s">
+        <v>4657</v>
+      </c>
+    </row>
+    <row r="134" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D134" s="10" t="s">
         <v>295</v>
       </c>
-    </row>
-    <row r="135" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K134" s="10" t="s">
+        <v>4658</v>
+      </c>
+    </row>
+    <row r="135" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D135" s="10" t="s">
         <v>296</v>
       </c>
-    </row>
-    <row r="136" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K135" s="10" t="s">
+        <v>4659</v>
+      </c>
+    </row>
+    <row r="136" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D136" s="10" t="s">
         <v>297</v>
       </c>
-    </row>
-    <row r="137" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K136" s="10" t="s">
+        <v>4660</v>
+      </c>
+    </row>
+    <row r="137" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D137" s="10" t="s">
         <v>298</v>
       </c>
-    </row>
-    <row r="138" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K137" s="10" t="s">
+        <v>4661</v>
+      </c>
+    </row>
+    <row r="138" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D138" s="10" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="139" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K138" s="10" t="s">
+        <v>4662</v>
+      </c>
+    </row>
+    <row r="139" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D139" s="10" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="140" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K139" s="10" t="s">
+        <v>4663</v>
+      </c>
+    </row>
+    <row r="140" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D140" s="10" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="141" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K140" s="10" t="s">
+        <v>4664</v>
+      </c>
+    </row>
+    <row r="141" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D141" s="10" t="s">
         <v>302</v>
       </c>
-    </row>
-    <row r="142" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K141" s="10" t="s">
+        <v>4665</v>
+      </c>
+    </row>
+    <row r="142" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D142" s="10" t="s">
         <v>303</v>
       </c>
-    </row>
-    <row r="143" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K142" s="10" t="s">
+        <v>4666</v>
+      </c>
+    </row>
+    <row r="143" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D143" s="10" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="144" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K143" s="10" t="s">
+        <v>4667</v>
+      </c>
+    </row>
+    <row r="144" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D144" s="10" t="s">
         <v>305</v>
       </c>
-    </row>
-    <row r="145" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K144" s="10" t="s">
+        <v>4668</v>
+      </c>
+    </row>
+    <row r="145" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D145" s="10" t="s">
         <v>306</v>
       </c>
-    </row>
-    <row r="146" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K145" s="10" t="s">
+        <v>4669</v>
+      </c>
+    </row>
+    <row r="146" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D146" s="10" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="147" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K146" s="10" t="s">
+        <v>4670</v>
+      </c>
+    </row>
+    <row r="147" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D147" s="10" t="s">
         <v>308</v>
       </c>
-    </row>
-    <row r="148" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K147" s="10" t="s">
+        <v>4671</v>
+      </c>
+    </row>
+    <row r="148" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D148" s="10" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="149" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K148" s="10" t="s">
+        <v>4672</v>
+      </c>
+    </row>
+    <row r="149" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D149" s="10" t="s">
         <v>311</v>
       </c>
-    </row>
-    <row r="150" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K149" s="10" t="s">
+        <v>4673</v>
+      </c>
+    </row>
+    <row r="150" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D150" s="10" t="s">
         <v>312</v>
       </c>
-    </row>
-    <row r="151" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K150" s="10" t="s">
+        <v>4674</v>
+      </c>
+    </row>
+    <row r="151" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D151" s="10" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="152" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K151" s="10" t="s">
+        <v>4675</v>
+      </c>
+    </row>
+    <row r="152" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D152" s="10" t="s">
         <v>314</v>
       </c>
-    </row>
-    <row r="153" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K152" s="10" t="s">
+        <v>4676</v>
+      </c>
+    </row>
+    <row r="153" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D153" s="10" t="s">
         <v>315</v>
       </c>
-    </row>
-    <row r="154" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K153" s="10" t="s">
+        <v>4677</v>
+      </c>
+    </row>
+    <row r="154" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D154" s="10" t="s">
         <v>316</v>
       </c>
-    </row>
-    <row r="155" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K154" s="10" t="s">
+        <v>4678</v>
+      </c>
+    </row>
+    <row r="155" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D155" s="10" t="s">
         <v>317</v>
       </c>
-    </row>
-    <row r="156" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K155" s="10" t="s">
+        <v>4679</v>
+      </c>
+    </row>
+    <row r="156" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D156" s="10" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="157" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K156" s="10" t="s">
+        <v>4680</v>
+      </c>
+    </row>
+    <row r="157" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D157" s="10" t="s">
         <v>319</v>
       </c>
-    </row>
-    <row r="158" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K157" s="10" t="s">
+        <v>4681</v>
+      </c>
+    </row>
+    <row r="158" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D158" s="10" t="s">
         <v>320</v>
       </c>
-    </row>
-    <row r="159" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K158" s="10" t="s">
+        <v>4682</v>
+      </c>
+    </row>
+    <row r="159" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D159" s="10" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="160" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K159" s="10" t="s">
+        <v>4683</v>
+      </c>
+    </row>
+    <row r="160" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D160" s="10" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="161" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K160" s="10" t="s">
+        <v>4684</v>
+      </c>
+    </row>
+    <row r="161" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D161" s="10" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="162" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K161" s="10" t="s">
+        <v>4685</v>
+      </c>
+    </row>
+    <row r="162" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D162" s="10" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="163" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K162" s="10" t="s">
+        <v>4686</v>
+      </c>
+    </row>
+    <row r="163" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D163" s="10" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="164" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K163" s="10" t="s">
+        <v>4687</v>
+      </c>
+    </row>
+    <row r="164" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D164" s="10" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="165" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K164" s="10" t="s">
+        <v>4688</v>
+      </c>
+    </row>
+    <row r="165" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D165" s="10" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="166" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K165" s="10" t="s">
+        <v>4689</v>
+      </c>
+    </row>
+    <row r="166" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D166" s="10" t="s">
         <v>4506</v>
       </c>
-    </row>
-    <row r="167" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="K166" s="10" t="s">
+        <v>4690</v>
+      </c>
+    </row>
+    <row r="167" spans="4:11" x14ac:dyDescent="0.25">
       <c r="D167" s="10" t="s">
         <v>4528</v>
+      </c>
+      <c r="K167" s="10" t="s">
+        <v>4691</v>
+      </c>
+    </row>
+    <row r="168" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D168" s="26"/>
+      <c r="K168" s="10" t="s">
+        <v>4692</v>
+      </c>
+    </row>
+    <row r="169" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D169" s="26"/>
+      <c r="K169" s="10" t="s">
+        <v>4693</v>
+      </c>
+    </row>
+    <row r="170" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D170" s="26"/>
+      <c r="K170" s="10" t="s">
+        <v>4694</v>
+      </c>
+    </row>
+    <row r="171" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D171" s="26"/>
+      <c r="K171" s="10" t="s">
+        <v>4695</v>
+      </c>
+    </row>
+    <row r="172" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D172" s="26"/>
+      <c r="K172" s="10" t="s">
+        <v>4696</v>
+      </c>
+    </row>
+    <row r="173" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D173" s="26"/>
+      <c r="K173" s="10" t="s">
+        <v>4697</v>
+      </c>
+    </row>
+    <row r="174" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D174" s="26"/>
+      <c r="K174" s="10" t="s">
+        <v>4698</v>
+      </c>
+    </row>
+    <row r="175" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D175" s="26"/>
+      <c r="K175" s="10" t="s">
+        <v>4699</v>
+      </c>
+    </row>
+    <row r="176" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D176" s="26"/>
+      <c r="K176" s="10" t="s">
+        <v>4700</v>
+      </c>
+    </row>
+    <row r="177" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D177" s="26"/>
+      <c r="K177" s="10" t="s">
+        <v>4701</v>
+      </c>
+    </row>
+    <row r="178" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D178" s="26"/>
+      <c r="K178" s="10" t="s">
+        <v>4702</v>
+      </c>
+    </row>
+    <row r="179" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D179" s="26"/>
+      <c r="K179" s="10" t="s">
+        <v>4703</v>
+      </c>
+    </row>
+    <row r="180" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D180" s="26"/>
+      <c r="K180" s="10" t="s">
+        <v>4704</v>
+      </c>
+    </row>
+    <row r="181" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D181" s="26"/>
+      <c r="K181" s="10" t="s">
+        <v>4705</v>
+      </c>
+    </row>
+    <row r="182" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D182" s="26"/>
+      <c r="K182" s="10" t="s">
+        <v>4706</v>
+      </c>
+    </row>
+    <row r="183" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D183" s="26"/>
+      <c r="K183" s="10" t="s">
+        <v>4707</v>
+      </c>
+    </row>
+    <row r="184" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D184" s="26"/>
+      <c r="K184" s="10" t="s">
+        <v>4708</v>
+      </c>
+    </row>
+    <row r="185" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D185" s="26"/>
+      <c r="K185" s="10" t="s">
+        <v>4709</v>
+      </c>
+    </row>
+    <row r="186" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D186" s="26"/>
+      <c r="K186" s="10" t="s">
+        <v>4710</v>
+      </c>
+    </row>
+    <row r="187" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D187" s="26"/>
+      <c r="K187" s="10" t="s">
+        <v>4711</v>
+      </c>
+    </row>
+    <row r="188" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D188" s="26"/>
+      <c r="K188" s="10" t="s">
+        <v>4712</v>
+      </c>
+    </row>
+    <row r="189" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D189" s="26"/>
+      <c r="K189" s="10" t="s">
+        <v>4713</v>
+      </c>
+    </row>
+    <row r="190" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D190" s="26"/>
+      <c r="K190" s="10" t="s">
+        <v>4714</v>
+      </c>
+    </row>
+    <row r="191" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D191" s="26"/>
+      <c r="K191" s="10" t="s">
+        <v>4715</v>
+      </c>
+    </row>
+    <row r="192" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D192" s="26"/>
+      <c r="K192" s="10" t="s">
+        <v>4716</v>
+      </c>
+    </row>
+    <row r="193" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D193" s="26"/>
+      <c r="K193" s="10" t="s">
+        <v>4717</v>
+      </c>
+    </row>
+    <row r="194" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D194" s="26"/>
+      <c r="K194" s="10" t="s">
+        <v>4718</v>
+      </c>
+    </row>
+    <row r="195" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D195" s="26"/>
+      <c r="K195" s="10" t="s">
+        <v>4719</v>
+      </c>
+    </row>
+    <row r="196" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D196" s="26"/>
+      <c r="K196" s="10" t="s">
+        <v>4720</v>
+      </c>
+    </row>
+    <row r="197" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D197" s="26"/>
+      <c r="K197" s="10" t="s">
+        <v>4721</v>
+      </c>
+    </row>
+    <row r="198" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D198" s="26"/>
+      <c r="K198" s="10" t="s">
+        <v>4722</v>
+      </c>
+    </row>
+    <row r="199" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D199" s="26"/>
+      <c r="K199" s="10" t="s">
+        <v>4723</v>
+      </c>
+    </row>
+    <row r="200" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D200" s="26"/>
+      <c r="K200" s="10" t="s">
+        <v>4724</v>
+      </c>
+    </row>
+    <row r="201" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D201" s="26"/>
+      <c r="K201" s="10" t="s">
+        <v>4725</v>
+      </c>
+    </row>
+    <row r="202" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D202" s="26"/>
+      <c r="K202" s="10" t="s">
+        <v>4726</v>
+      </c>
+    </row>
+    <row r="203" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D203" s="26"/>
+      <c r="K203" s="10" t="s">
+        <v>4727</v>
+      </c>
+    </row>
+    <row r="204" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D204" s="26"/>
+      <c r="K204" s="10" t="s">
+        <v>4728</v>
+      </c>
+    </row>
+    <row r="205" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D205" s="26"/>
+      <c r="K205" s="10" t="s">
+        <v>4729</v>
+      </c>
+    </row>
+    <row r="206" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D206" s="26"/>
+      <c r="K206" s="10" t="s">
+        <v>4730</v>
+      </c>
+    </row>
+    <row r="207" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D207" s="26"/>
+      <c r="K207" s="10" t="s">
+        <v>4731</v>
+      </c>
+    </row>
+    <row r="208" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D208" s="26"/>
+      <c r="K208" s="10" t="s">
+        <v>4732</v>
+      </c>
+    </row>
+    <row r="209" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D209" s="26"/>
+      <c r="K209" s="10" t="s">
+        <v>4733</v>
+      </c>
+    </row>
+    <row r="210" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D210" s="26"/>
+      <c r="K210" s="10" t="s">
+        <v>4734</v>
+      </c>
+    </row>
+    <row r="211" spans="4:11" x14ac:dyDescent="0.25">
+      <c r="D211" s="26"/>
+      <c r="K211" s="26" t="s">
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>